<commit_message>
fix(questions): relabel prioritisation answers so they cannot read as risk
A tester picked every "Low" prioritisation answer believing it was the safe
choice. Low/Medium/High now become descriptive labels (Heavy/Moderate/Light
usage, Simple/Moderately/Very complex, Ready/Partly ready/Not ready), with
the most AI-ready answer listed first. Option ids are unchanged, so saved
registers still load. The block adds a note: these are not risk questions.
Templates are regenerated from the same data.
</commit_message>
<xml_diff>
--- a/public/templates/ar/impact-assessment.xlsx
+++ b/public/templates/ar/impact-assessment.xlsx
@@ -754,7 +754,7 @@
         <v>ما كثافة استخدام الخدمة؟</v>
       </c>
       <c r="C21" t="str">
-        <v>منخفضة: استخدام محدود ومعاملات غير متكررة; متوسطة; مرتفعة: استخدام واسع ومعاملات متكررة</v>
+        <v>كثيفة: استخدام واسع ومعاملات متكررة; معتدلة; محدودة: استخدام محدود ومعاملات غير متكررة</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -771,7 +771,7 @@
         <v>ما مستوى تعقيد تنفيذ الخدمة أو تحويلها؟</v>
       </c>
       <c r="C22" t="str">
-        <v>منخفض: بسيط وموحّد وقابل للتكرار; متوسط; مرتفع: متعدد الجهات ومتغيّر وخاضع لحوكمة مشددة</v>
+        <v>بسيط: موحّد وقابل للتكرار; معقّد إلى حدٍّ ما; شديد التعقيد: متعدد الجهات ومتغيّر وخاضع لحوكمة مشددة</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -788,7 +788,7 @@
         <v>ما مدى جاهزية الخدمة لتبنّي الذكاء الاصطناعي؟</v>
       </c>
       <c r="C23" t="str">
-        <v>منخفضة: يدوية ومجزأة وغير واضحة; متوسطة; مرتفعة: منظّمة ورقمية ومتكاملة</v>
+        <v>جاهزة (رقمية ومتكاملة); جاهزة جزئياً; غير جاهزة (يدوية ومجزأة)</v>
       </c>
       <c r="D23" t="str">
         <v/>

</xml_diff>

<commit_message>
feat(tier): explain where the tier comes from and mark optional sections
A tester skipped the optional sections, saw a High tier and assumed the two
were linked. The tier card now says the tier comes from the 8 quick-check
questions and that skipping the optional sections never raises it. The
deep-dive and prioritisation headers carry an Optional badge.
</commit_message>
<xml_diff>
--- a/public/templates/ar/impact-assessment.xlsx
+++ b/public/templates/ar/impact-assessment.xlsx
@@ -748,7 +748,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>تحديد الأولوية للذكاء الاصطناعي (اختياري)</v>
+        <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B21" t="str">
         <v>ما كثافة استخدام الخدمة؟</v>
@@ -765,7 +765,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>تحديد الأولوية للذكاء الاصطناعي (اختياري)</v>
+        <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B22" t="str">
         <v>ما مستوى تعقيد تنفيذ الخدمة أو تحويلها؟</v>
@@ -782,7 +782,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>تحديد الأولوية للذكاء الاصطناعي (اختياري)</v>
+        <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B23" t="str">
         <v>ما مدى جاهزية الخدمة لتبنّي الذكاء الاصطناعي؟</v>

</xml_diff>

<commit_message>
feat(questions): ask first whether the solution uses AI when it runs
A tester's product was built with AI coding tools but has no AI inside, and
the kit still forced a risk tier. The quick check now opens with a scope
question. Answering No shows that AI governance controls don't apply, plus
general software quality and security pointers, and no tier. The question
carries no points and an unanswered one counts as in scope, so saved
registers keep their tiers. The register shows "No AI at runtime" and the
register template gains a runtime_ai column. See ADR 007.
</commit_message>
<xml_diff>
--- a/public/templates/ar/impact-assessment.xlsx
+++ b/public/templates/ar/impact-assessment.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="52.83203125" customWidth="1"/>
@@ -442,13 +442,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>الفحص السريع</v>
+        <v>النطاق</v>
       </c>
       <c r="B3" t="str">
-        <v>على ماذا تؤثر مخرجات نظام الذكاء الاصطناعي؟</v>
+        <v>هل يستخدم الحل الذكاء الاصطناعي أثناء تشغيله؟</v>
       </c>
       <c r="C3" t="str">
-        <v>الإنتاجية الداخلية فقط (مسودات، ملخصات، بحث) (0); معلومات تُقدَّم للجمهور أو المتعاملين (5); توصيات للموظفين بشأن أشخاص بعينهم (15); قرارات تمس حقوق الأفراد أو مستحقاتهم أو وصولهم إلى الخدمات أو أموالهم (25); التصنيف الاجتماعي للأفراد، أو التلاعب بالسلوك، أو المراقبة البيومترية الفورية للجمهور (0)</v>
+        <v>نعم: يستخدم نموذجاً أو خدمة ذكاء اصطناعي أثناء التشغيل; لا: استُخدم الذكاء الاصطناعي في بنائه فقط، أو لم يُستخدم إطلاقاً</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -462,10 +462,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B4" t="str">
-        <v>ما البيانات التي يستخدمها؟</v>
+        <v>على ماذا تؤثر مخرجات نظام الذكاء الاصطناعي؟</v>
       </c>
       <c r="C4" t="str">
-        <v>لا بيانات عن الأشخاص، أو بيانات عامة فقط (0); بيانات عمل داخلية دون بيانات شخصية (3); بيانات شخصية (10); بيانات شخصية حساسة (18)</v>
+        <v>الإنتاجية الداخلية فقط (مسودات، ملخصات، بحث) (0); معلومات تُقدَّم للجمهور أو المتعاملين (5); توصيات للموظفين بشأن أشخاص بعينهم (15); قرارات تمس حقوق الأفراد أو مستحقاتهم أو وصولهم إلى الخدمات أو أموالهم (25); التصنيف الاجتماعي للأفراد، أو التلاعب بالسلوك، أو المراقبة البيومترية الفورية للجمهور (0)</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -479,10 +479,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B5" t="str">
-        <v>من قد يتأثر؟</v>
+        <v>ما البيانات التي يستخدمها؟</v>
       </c>
       <c r="C5" t="str">
-        <v>الموظفون فقط (3); المتعاملون أو الجمهور (8); فئات أكثر عرضة للتأثر (الأطفال، كبار السن، أصحاب الهمم) (15)</v>
+        <v>لا بيانات عن الأشخاص، أو بيانات عامة فقط (0); بيانات عمل داخلية دون بيانات شخصية (3); بيانات شخصية (10); بيانات شخصية حساسة (18)</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -496,10 +496,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B6" t="str">
-        <v>ما نوع الذكاء الاصطناعي المستخدم؟</v>
+        <v>من قد يتأثر؟</v>
       </c>
       <c r="C6" t="str">
-        <v>تنبؤي (يقيّم أو يصنّف أو يتوقع) (5); توليدي (يُنتج نصوصاً أو صوراً أو إجابات) (5); وكيلي (يخطط وينفّذ إجراءات) (10)</v>
+        <v>الموظفون فقط (3); المتعاملون أو الجمهور (8); فئات أكثر عرضة للتأثر (الأطفال، كبار السن، أصحاب الهمم) (15)</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -513,10 +513,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B7" t="str">
-        <v>إلى أي مدى يعمل باستقلالية؟</v>
+        <v>ما نوع الذكاء الاصطناعي المستخدم؟</v>
       </c>
       <c r="C7" t="str">
-        <v>يقترح فقط؛ والإنسان يقرر وينفّذ (0); ينفّذ فقط بعد موافقة الإنسان (5); ينفّذ من تلقاء نفسه مع متابعة بشرية (15); مستقل تماماً دون تدخل بشري معتاد (25)</v>
+        <v>تنبؤي (يقيّم أو يصنّف أو يتوقع) (5); توليدي (يُنتج نصوصاً أو صوراً أو إجابات) (5); وكيلي (يخطط وينفّذ إجراءات) (10)</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -530,10 +530,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B8" t="str">
-        <v>كيف يراجع البشر عمله؟</v>
+        <v>إلى أي مدى يعمل باستقلالية؟</v>
       </c>
       <c r="C8" t="str">
-        <v>يراجع شخصٌ كل مُخرج (0); مراجعة عينات أو الحالات الاستثنائية (5); فقط عند ورود شكوى (12); لا توجد مراجعة معتادة (20)</v>
+        <v>يقترح فقط؛ والإنسان يقرر وينفّذ (0); ينفّذ فقط بعد موافقة الإنسان (5); ينفّذ من تلقاء نفسه مع متابعة بشرية (15); مستقل تماماً دون تدخل بشري معتاد (25)</v>
       </c>
       <c r="D8" t="str">
         <v/>
@@ -547,10 +547,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B9" t="str">
-        <v>ما الذي يمكنه تغييره في الأنظمة الأخرى؟</v>
+        <v>كيف يراجع البشر عمله؟</v>
       </c>
       <c r="C9" t="str">
-        <v>لا شيء: لا صلاحيات أو قراءة فقط (0); يكتب في أدوات داخلية غير حرجة (8); يكتب في أنظمة السجل، أو يجري مدفوعات، أو يرسل رسائل خارجية (15)</v>
+        <v>يراجع شخصٌ كل مُخرج (0); مراجعة عينات أو الحالات الاستثنائية (5); فقط عند ورود شكوى (12); لا توجد مراجعة معتادة (20)</v>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -564,10 +564,10 @@
         <v>الفحص السريع</v>
       </c>
       <c r="B10" t="str">
-        <v>إذا أخطأ، هل يمكن التراجع عن النتيجة؟</v>
+        <v>ما الذي يمكنه تغييره في الأنظمة الأخرى؟</v>
       </c>
       <c r="C10" t="str">
-        <v>نعم، بسهولة (0); نعم، ولكن بجهد (6); لا، أو فقط مع ضرر دائم (15)</v>
+        <v>لا شيء: لا صلاحيات أو قراءة فقط (0); يكتب في أدوات داخلية غير حرجة (8); يكتب في أنظمة السجل، أو يجري مدفوعات، أو يرسل رسائل خارجية (15)</v>
       </c>
       <c r="D10" t="str">
         <v/>
@@ -578,13 +578,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>التقييم المعمّق</v>
+        <v>الفحص السريع</v>
       </c>
       <c r="B11" t="str">
-        <v>كم عدد الأشخاص الذين يتأثرون به شهرياً؟</v>
+        <v>إذا أخطأ، هل يمكن التراجع عن النتيجة؟</v>
       </c>
       <c r="C11" t="str">
-        <v>أقل من 1,000 (0); من 1,000 إلى 100,000 (4); أكثر من 100,000 (8)</v>
+        <v>نعم، بسهولة (0); نعم، ولكن بجهد (6); لا، أو فقط مع ضرر دائم (15)</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -598,10 +598,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B12" t="str">
-        <v>هل يمكنك شرح نتيجة بعينها للشخص المتأثر بها؟</v>
+        <v>كم عدد الأشخاص الذين يتأثرون به شهرياً؟</v>
       </c>
       <c r="C12" t="str">
-        <v>نعم، بلغة واضحة (0); جزئياً (4); لا (8)</v>
+        <v>أقل من 1,000 (0); من 1,000 إلى 100,000 (4); أكثر من 100,000 (8)</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -615,10 +615,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B13" t="str">
-        <v>هل يعتمد على نموذج أو خدمة من طرف ثالث؟</v>
+        <v>هل يمكنك شرح نتيجة بعينها للشخص المتأثر بها؟</v>
       </c>
       <c r="C13" t="str">
-        <v>لا، مطوَّر ومستضاف داخلياً (0); نعم، مستضاف داخل الدولة وتحت سيطرتنا (3); نعم، خدمة خارجية خارج سيطرتنا (6)</v>
+        <v>نعم، بلغة واضحة (0); جزئياً (4); لا (8)</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -632,10 +632,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B14" t="str">
-        <v>هل تنتقل البيانات خارج الدولة؟</v>
+        <v>هل يعتمد على نموذج أو خدمة من طرف ثالث؟</v>
       </c>
       <c r="C14" t="str">
-        <v>لا (0); غير متأكد (4); نعم (6)</v>
+        <v>لا، مطوَّر ومستضاف داخلياً (0); نعم، مستضاف داخل الدولة وتحت سيطرتنا (3); نعم، خدمة خارجية خارج سيطرتنا (6)</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -649,10 +649,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B15" t="str">
-        <v>هل اختُبر للتأكد من عدم تحيّز نتائجه بين الفئات المختلفة؟</v>
+        <v>هل تنتقل البيانات خارج الدولة؟</v>
       </c>
       <c r="C15" t="str">
-        <v>نعم، بنتائج موثّقة (0); مخطط له ولم يُنفَّذ بعد (4); لا (8)</v>
+        <v>لا (0); غير متأكد (4); نعم (6)</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -666,10 +666,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B16" t="str">
-        <v>هل اختُبر ضد إساءة الاستخدام والهجمات (مثل حقن التعليمات)؟</v>
+        <v>هل اختُبر للتأكد من عدم تحيّز نتائجه بين الفئات المختلفة؟</v>
       </c>
       <c r="C16" t="str">
-        <v>نعم (0); مخطط له (4); لا (8)</v>
+        <v>نعم، بنتائج موثّقة (0); مخطط له ولم يُنفَّذ بعد (4); لا (8)</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -683,10 +683,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B17" t="str">
-        <v>هل يُراقَب أداؤه بعد الإطلاق؟</v>
+        <v>هل اختُبر ضد إساءة الاستخدام والهجمات (مثل حقن التعليمات)؟</v>
       </c>
       <c r="C17" t="str">
-        <v>نعم، بمؤشرات ومسؤولين محددين (0); بشكل غير منتظم (4); لا (8)</v>
+        <v>نعم (0); مخطط له (4); لا (8)</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -700,10 +700,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B18" t="str">
-        <v>هل توجد آلية لإيقافه ومعالجة الحوادث؟</v>
+        <v>هل يُراقَب أداؤه بعد الإطلاق؟</v>
       </c>
       <c r="C18" t="str">
-        <v>نعم، موثّقة ومختبرة (0); جزئياً (4); لا (8)</v>
+        <v>نعم، بمؤشرات ومسؤولين محددين (0); بشكل غير منتظم (4); لا (8)</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -717,10 +717,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B19" t="str">
-        <v>هل يُستخدم في مجال خاضع للتنظيم؟</v>
+        <v>هل توجد آلية لإيقافه ومعالجة الحوادث؟</v>
       </c>
       <c r="C19" t="str">
-        <v>لا (0); نعم (6)</v>
+        <v>نعم، موثّقة ومختبرة (0); جزئياً (4); لا (8)</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -734,10 +734,10 @@
         <v>التقييم المعمّق</v>
       </c>
       <c r="B20" t="str">
-        <v>هل يُبلَّغ الأشخاص بأنهم يتعاملون مع ذكاء اصطناعي؟</v>
+        <v>هل يُستخدم في مجال خاضع للتنظيم؟</v>
       </c>
       <c r="C20" t="str">
-        <v>نعم، بوضوح (0); لا (5)</v>
+        <v>لا (0); نعم (6)</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -748,13 +748,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>تحديد الأولوية للذكاء الاصطناعي</v>
+        <v>التقييم المعمّق</v>
       </c>
       <c r="B21" t="str">
-        <v>ما كثافة استخدام الخدمة؟</v>
+        <v>هل يُبلَّغ الأشخاص بأنهم يتعاملون مع ذكاء اصطناعي؟</v>
       </c>
       <c r="C21" t="str">
-        <v>كثيفة: استخدام واسع ومعاملات متكررة; معتدلة; محدودة: استخدام محدود ومعاملات غير متكررة</v>
+        <v>نعم، بوضوح (0); لا (5)</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -768,10 +768,10 @@
         <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B22" t="str">
-        <v>ما مستوى تعقيد تنفيذ الخدمة أو تحويلها؟</v>
+        <v>ما كثافة استخدام الخدمة؟</v>
       </c>
       <c r="C22" t="str">
-        <v>بسيط: موحّد وقابل للتكرار; معقّد إلى حدٍّ ما; شديد التعقيد: متعدد الجهات ومتغيّر وخاضع لحوكمة مشددة</v>
+        <v>كثيفة: استخدام واسع ومعاملات متكررة; معتدلة; محدودة: استخدام محدود ومعاملات غير متكررة</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -785,10 +785,10 @@
         <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B23" t="str">
-        <v>ما مدى جاهزية الخدمة لتبنّي الذكاء الاصطناعي؟</v>
+        <v>ما مستوى تعقيد تنفيذ الخدمة أو تحويلها؟</v>
       </c>
       <c r="C23" t="str">
-        <v>جاهزة (رقمية ومتكاملة); جاهزة جزئياً; غير جاهزة (يدوية ومجزأة)</v>
+        <v>بسيط: موحّد وقابل للتكرار; معقّد إلى حدٍّ ما; شديد التعقيد: متعدد الجهات ومتغيّر وخاضع لحوكمة مشددة</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -799,13 +799,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v/>
+        <v>تحديد الأولوية للذكاء الاصطناعي</v>
       </c>
       <c r="B24" t="str">
-        <v/>
+        <v>ما مدى جاهزية الخدمة لتبنّي الذكاء الاصطناعي؟</v>
       </c>
       <c r="C24" t="str">
-        <v/>
+        <v>جاهزة (رقمية ومتكاملة); جاهزة جزئياً; غير جاهزة (يدوية ومجزأة)</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -819,7 +819,7 @@
         <v/>
       </c>
       <c r="B25" t="str">
-        <v>المستوى الناتج</v>
+        <v/>
       </c>
       <c r="C25" t="str">
         <v/>
@@ -836,7 +836,7 @@
         <v/>
       </c>
       <c r="B26" t="str">
-        <v>الأسباب</v>
+        <v>المستوى الناتج</v>
       </c>
       <c r="C26" t="str">
         <v/>
@@ -853,7 +853,7 @@
         <v/>
       </c>
       <c r="B27" t="str">
-        <v>الاعتماد</v>
+        <v>الأسباب</v>
       </c>
       <c r="C27" t="str">
         <v/>
@@ -870,7 +870,7 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>أعدّه</v>
+        <v>الاعتماد</v>
       </c>
       <c r="C28" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v/>
       </c>
       <c r="B29" t="str">
-        <v>راجعه</v>
+        <v>أعدّه</v>
       </c>
       <c r="C29" t="str">
         <v/>
@@ -904,7 +904,7 @@
         <v/>
       </c>
       <c r="B30" t="str">
-        <v>القرار</v>
+        <v>راجعه</v>
       </c>
       <c r="C30" t="str">
         <v/>
@@ -921,21 +921,38 @@
         <v/>
       </c>
       <c r="B31" t="str">
+        <v>القرار</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+      <c r="B32" t="str">
         <v>التاريخ</v>
       </c>
-      <c r="C31" t="str">
-        <v/>
-      </c>
-      <c r="D31" t="str">
-        <v/>
-      </c>
-      <c r="E31" t="str">
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>